<commit_message>
Update data and source file
</commit_message>
<xml_diff>
--- a/花开富贵.xlsx
+++ b/花开富贵.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18060" windowHeight="15500"/>
+    <workbookView windowWidth="23420" windowHeight="15500"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -35,43 +35,43 @@
     <t>魔力卡花匠</t>
   </si>
   <si>
-    <t>蓝铁，幻紫、紫麦冬花、雾粉麦冬花、粉白君子兰、嫣红杜鹃花</t>
+    <t>蓝叶苏铁，幻紫铁线莲、紫麦冬花、雾粉麦冬花、粉白君子兰、嫣红杜鹃</t>
   </si>
   <si>
     <t>董沅芹</t>
   </si>
   <si>
-    <t>蓝铁、赤焰、珠宝之心</t>
+    <t>蓝叶苏铁、赤焰火焰兰、珠宝之心</t>
   </si>
   <si>
     <t>耶律姝艳</t>
   </si>
   <si>
-    <t>粉色满天星14，玫红非洲堇14，鸳鸯茉莉，绿铁，浅黄绿绒蒿，幽兰绿绒蒿，正红大丽花，薄粉蕙兰，淡茜蜀葵花，三色络新妇，杏黄杜鹃，紫粉矢车菊，香槟玫瑰，明黄跳舞兰，绯色腊梅，梦紫郁金香</t>
+    <t>粉色满天星，玫红非洲堇，鸳鸯茉莉，绿叶苏铁，浅黄绿绒蒿，幽兰绿绒蒿，正红大丽花，薄粉蕙兰，淡茜蜀葵花，杏黄杜鹃、紫矢车菊、粉矢车菊、香槟玫瑰，明黄跳舞兰，绯色腊梅，梦紫郁金香</t>
   </si>
   <si>
     <t>长孙若微</t>
   </si>
   <si>
-    <t>殷红灯笼花，白花马齿笕，嫩黄马齿笕，蓝色满天星，粉蓝紫矢车菊，浅蓝紫红落新妇，绿铁，蓝色牵牛花浅粉夹竹桃</t>
+    <t>殷红灯笼花，白花马齿笕，嫩黄马齿笕，蓝色满天星，紫矢车菊、粉矢车菊、蓝矢车菊，绿叶苏铁，蓝色牵牛花，浅粉夹竹桃</t>
   </si>
   <si>
     <t>大稻</t>
   </si>
   <si>
-    <t>蓝面花、钢丝球、鹅黄铁筷花，朱柿长寿花，绯色腊梅、</t>
+    <t>澄蓝龙面花、葡萄紫牡丹球、鹅黄铁筷花，朱柿长寿花，绯色腊梅、伯利恒之星、碧落月见草、绛粉大岩桐</t>
   </si>
   <si>
     <t>慕蕊</t>
   </si>
   <si>
-    <t>浅韵美女樱、粉鹤、紫美人、紫葱、伯利恒之星、红/白垂筒花、柔紫石斛兰、紫荷包牡丹、三色车菊、忽地笑、杏白忘忧草、淡粉马齿苋、银白翠竹、正红大丽花、月白格桑花、三色落新妇、淡茜蜀葵花、曼陀罗化、星河、金蝉腰、粉樱月见草、碧落月见草、绯色腊梅、藤黄露薇花、莹白露薇花、粉/白谷鸢尾花</t>
+    <t>浅韵美女樱、粉鹤芋、黛紫紫美人、轻紫大花葱、伯利恒之星、橘红垂筒花、霜白垂筒花、柔紫石斛兰、紫荷包牡丹、紫矢车菊、粉矢车菊、蓝矢车菊、忽地笑、杏白忘忧草、淡粉马齿苋、银白翠珠、正红大丽花、月白格桑花、淡茜蜀葵花、曼陀罗花、星河映蕊、金缠腰、粉樱月见草、碧落月见草、绯色腊梅、藤黄露薇花、莹白露薇花、霜白谷鸢尾花、冰蓝谷鸢尾</t>
   </si>
   <si>
     <t>暖香</t>
   </si>
   <si>
-    <t>曼莎珠华，鸳鸯茉莉、橙黄美人、粉鹤、伯利恒，绿铁，三色矢车菊，三色落新妇，三色垂筒花，浅橘/明黄如意菊，柔紫/碧白石斛兰，粉/白谷鸢尾，蓝/黄/粉牵牛，轻紫翠竹、丹紫夹竹桃</t>
+    <t>曼珠沙华，鸳鸯茉莉、橙黄虞美人、粉鹤芋、伯利恒之星，绿叶苏铁，紫矢车菊、粉矢车菊、蓝矢车菊、霜白垂筒花、橘红垂筒花、明黄垂筒花、浅橘如意菊、明黄如意菊，柔紫石斛兰、碧白石斛兰，桃粉谷鸢尾、霜白谷鸢尾，冰蓝矮牵牛、明黄矮牵牛、淡粉矮牵牛，轻紫翠珠、丹紫夹竹桃</t>
   </si>
   <si>
     <t>绿豆</t>
@@ -80,13 +80,13 @@
     <t>千婷</t>
   </si>
   <si>
-    <t>绿铁、蓝色满天星</t>
+    <t>绿叶苏铁、蓝色满天星</t>
   </si>
   <si>
     <t>丧彪</t>
   </si>
   <si>
-    <t xml:space="preserve">黑曜大丽花 浅紫落新妇  浅蓝络新妇  蓝色牵牛花 
+    <t xml:space="preserve">黑曜大丽花 冰蓝矮牵牛
 </t>
   </si>
   <si>
@@ -99,13 +99,13 @@
     <t>嘉文</t>
   </si>
   <si>
-    <t>轻紫翠竹、金盏蜀葵花</t>
+    <t>轻紫翠珠、金盏蜀葵花</t>
   </si>
   <si>
     <t>上官雁</t>
   </si>
   <si>
-    <t>粉紫华珊、香槟玫瑰、鸳鸯茉莉，木槿花、冬青、紫郁金香、冰蓝矮牵牛、淡茜蜀葵花、月白格桑花</t>
+    <t>粉紫华珊、香槟玫瑰、鸳鸯茉莉，粉红木槿花、轮生冬青、梦紫郁金香、冰蓝矮牵牛、淡茜蜀葵花、月白格桑花</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1286,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1" spans="1:2">
+    <row r="4" ht="116" customHeight="1" spans="1:2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" spans="1:2">
+    <row r="5" ht="125" customHeight="1" spans="1:2">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="51" customHeight="1" spans="1:2">
+    <row r="6" ht="129" customHeight="1" spans="1:2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="62.25" customHeight="1" spans="1:2">
+    <row r="7" ht="232" customHeight="1" spans="1:2">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="49.5" customHeight="1" spans="1:2">
+    <row r="8" ht="123" customHeight="1" spans="1:2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" ht="15.2" spans="1:2">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>22</v>
       </c>

</xml_diff>